<commit_message>
Did SQL analysis for 1st table
</commit_message>
<xml_diff>
--- a/Data/Processed 2020/1. Dim_Demographics_Employment.xlsx
+++ b/Data/Processed 2020/1. Dim_Demographics_Employment.xlsx
@@ -1,9 +1,9 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30305"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30317"/>
   <workbookPr defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="54" documentId="11_E60897F41BE170836B02CE998F75CCDC64E183C8" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D332AD65-E02A-4C15-9011-12557C7A3DE5}"/>
+  <xr:revisionPtr revIDLastSave="55" documentId="11_E60897F41BE170836B02CE998F75CCDC64E183C8" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{24815AFB-8E56-4E6F-9422-8C7900E28A81}"/>
   <bookViews>
     <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -946,7 +946,7 @@
   <dimension ref="A1:L1508"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelCol="1"/>
   <cols>
-    <col min="1" max="1" width="11.85546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="16.28515625" customWidth="1"/>
     <col min="2" max="2" width="24.85546875" bestFit="1" customWidth="1" outlineLevel="1"/>
     <col min="3" max="3" width="20.140625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="48.140625" bestFit="1" customWidth="1"/>

</xml_diff>